<commit_message>
location and ui changed
</commit_message>
<xml_diff>
--- a/public/TrackTrace_Project_Template.xlsx
+++ b/public/TrackTrace_Project_Template.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
   <si>
     <t xml:space="preserve">Item Name</t>
   </si>
@@ -62,6 +62,9 @@
   </si>
   <si>
     <t xml:space="preserve">Weight</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Custom Packing Group</t>
   </si>
 </sst>
 </file>
@@ -75,7 +78,7 @@
     <numFmt numFmtId="167" formatCode="0%"/>
     <numFmt numFmtId="168" formatCode="0.0"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="8">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -123,14 +126,6 @@
       <sz val="10"/>
       <color rgb="FFFFFFFF"/>
       <name val="Times New Roman"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <b val="true"/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
@@ -211,6 +206,10 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="24" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -225,10 +224,6 @@
     </xf>
     <xf numFmtId="168" fontId="6" fillId="2" borderId="0" xfId="24" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="24" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -479,59 +474,65 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:N1"/>
+  <dimension ref="A1:O1"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="38"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="11" min="5" style="1" width="11.53"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="12" style="1" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="12.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="16.02"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="14.62"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="17.62"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="10" min="5" style="1" width="11.53"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="8.41"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="8.5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="10.32"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="2" width="12.73"/>
   </cols>
   <sheetData>
-    <row r="1" s="6" customFormat="true" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+    <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="I1" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="J1" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="K1" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="5" t="s">
+      <c r="L1" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="4" t="s">
+      <c r="M1" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="4" t="s">
+      <c r="N1" s="5" t="s">
         <v>13</v>
+      </c>
+      <c r="O1" s="5" t="s">
+        <v>14</v>
       </c>
     </row>
   </sheetData>

</xml_diff>